<commit_message>
7. RANDOM FOREST 26_05_19
</commit_message>
<xml_diff>
--- a/outputs/Estadistica_L8_26_05_11/Estadisticas_L8_26_05_11.xlsx
+++ b/outputs/Estadistica_L8_26_05_11/Estadisticas_L8_26_05_11.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Maestria_Geomatica\Semestre_IV\Tesis_Python\Datos\TIFF\Estadistica_L8_26_05_11\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Equipo\Tesis\SemestreIV\Objetivo1\Objetivo1_26_02_20\outputs\Estadistica_L8_26_05_11\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2A82D2E-ECAE-48AD-96BE-E0910A2C8F46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B9E6156-B679-4865-8A7B-CE34619D8704}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -771,9 +771,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:AB331"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -861,7 +863,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -944,7 +946,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>28</v>
       </c>
@@ -1027,7 +1029,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>28</v>
       </c>
@@ -1110,7 +1112,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>28</v>
       </c>
@@ -1774,7 +1776,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="13" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>46</v>
       </c>
@@ -1857,7 +1859,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="14" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>46</v>
       </c>
@@ -1940,7 +1942,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="15" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>46</v>
       </c>
@@ -2023,7 +2025,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="16" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>46</v>
       </c>
@@ -2687,7 +2689,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="24" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>49</v>
       </c>
@@ -2770,7 +2772,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="25" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>49</v>
       </c>
@@ -2853,7 +2855,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="26" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>49</v>
       </c>
@@ -2936,7 +2938,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="27" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>49</v>
       </c>
@@ -3600,7 +3602,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="35" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>52</v>
       </c>
@@ -3683,7 +3685,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="36" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>52</v>
       </c>
@@ -3766,7 +3768,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="37" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>52</v>
       </c>
@@ -3849,7 +3851,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="38" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>52</v>
       </c>
@@ -4513,7 +4515,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="46" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>55</v>
       </c>
@@ -4596,7 +4598,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="47" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>55</v>
       </c>
@@ -4679,7 +4681,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="48" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>55</v>
       </c>
@@ -4762,7 +4764,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="49" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>55</v>
       </c>
@@ -5426,7 +5428,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="57" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>58</v>
       </c>
@@ -5509,7 +5511,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="58" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>58</v>
       </c>
@@ -5592,7 +5594,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="59" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>58</v>
       </c>
@@ -5675,7 +5677,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="60" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>58</v>
       </c>
@@ -6339,7 +6341,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="68" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>61</v>
       </c>
@@ -6422,7 +6424,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="69" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>61</v>
       </c>
@@ -6505,7 +6507,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="70" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>61</v>
       </c>
@@ -6588,7 +6590,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="71" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>61</v>
       </c>
@@ -7252,7 +7254,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="79" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>63</v>
       </c>
@@ -7335,7 +7337,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="80" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>63</v>
       </c>
@@ -7418,7 +7420,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="81" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>63</v>
       </c>
@@ -7501,7 +7503,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="82" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>63</v>
       </c>
@@ -8165,7 +8167,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="90" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>65</v>
       </c>
@@ -8248,7 +8250,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="91" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>65</v>
       </c>
@@ -8331,7 +8333,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="92" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>65</v>
       </c>
@@ -8414,7 +8416,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="93" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>65</v>
       </c>
@@ -9078,7 +9080,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="101" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>67</v>
       </c>
@@ -9161,7 +9163,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="102" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>67</v>
       </c>
@@ -9244,7 +9246,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="103" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>67</v>
       </c>
@@ -9327,7 +9329,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="104" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>67</v>
       </c>
@@ -9991,7 +9993,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="112" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>69</v>
       </c>
@@ -10074,7 +10076,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="113" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>69</v>
       </c>
@@ -10157,7 +10159,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="114" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>69</v>
       </c>
@@ -10240,7 +10242,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="115" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>69</v>
       </c>
@@ -10904,7 +10906,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="123" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>71</v>
       </c>
@@ -10987,7 +10989,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="124" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>71</v>
       </c>
@@ -11070,7 +11072,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="125" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>71</v>
       </c>
@@ -11153,7 +11155,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="126" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>71</v>
       </c>
@@ -11817,7 +11819,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="134" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>73</v>
       </c>
@@ -11900,7 +11902,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="135" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>73</v>
       </c>
@@ -11983,7 +11985,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="136" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>73</v>
       </c>
@@ -12066,7 +12068,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="137" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>73</v>
       </c>
@@ -12730,7 +12732,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="145" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>75</v>
       </c>
@@ -12813,7 +12815,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="146" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>75</v>
       </c>
@@ -12896,7 +12898,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="147" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>75</v>
       </c>
@@ -12979,7 +12981,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="148" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>75</v>
       </c>
@@ -13643,7 +13645,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="156" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>77</v>
       </c>
@@ -13726,7 +13728,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="157" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>77</v>
       </c>
@@ -13809,7 +13811,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="158" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>77</v>
       </c>
@@ -13892,7 +13894,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="159" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>77</v>
       </c>
@@ -14556,7 +14558,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="167" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>79</v>
       </c>
@@ -14639,7 +14641,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="168" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>79</v>
       </c>
@@ -14722,7 +14724,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="169" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>79</v>
       </c>
@@ -14805,7 +14807,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="170" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>79</v>
       </c>
@@ -15469,7 +15471,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="178" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>81</v>
       </c>
@@ -15552,7 +15554,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="179" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>81</v>
       </c>
@@ -15635,7 +15637,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="180" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>81</v>
       </c>
@@ -15718,7 +15720,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="181" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>81</v>
       </c>
@@ -16382,7 +16384,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="189" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>83</v>
       </c>
@@ -16465,7 +16467,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="190" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>83</v>
       </c>
@@ -16548,7 +16550,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="191" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>83</v>
       </c>
@@ -16631,7 +16633,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="192" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>83</v>
       </c>
@@ -17295,7 +17297,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="200" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>85</v>
       </c>
@@ -17378,7 +17380,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="201" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>85</v>
       </c>
@@ -17461,7 +17463,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="202" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>85</v>
       </c>
@@ -17544,7 +17546,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="203" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>85</v>
       </c>
@@ -18208,7 +18210,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="211" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>87</v>
       </c>
@@ -18291,7 +18293,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="212" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>87</v>
       </c>
@@ -18374,7 +18376,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="213" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>87</v>
       </c>
@@ -18457,7 +18459,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="214" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>87</v>
       </c>
@@ -19121,7 +19123,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="222" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>89</v>
       </c>
@@ -19204,7 +19206,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="223" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>89</v>
       </c>
@@ -19287,7 +19289,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="224" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>89</v>
       </c>
@@ -19370,7 +19372,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="225" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>89</v>
       </c>
@@ -20034,7 +20036,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="233" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
         <v>91</v>
       </c>
@@ -20117,7 +20119,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="234" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
         <v>91</v>
       </c>
@@ -20200,7 +20202,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="235" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
         <v>91</v>
       </c>
@@ -20283,7 +20285,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="236" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
         <v>91</v>
       </c>
@@ -20947,7 +20949,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="244" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>93</v>
       </c>
@@ -21030,7 +21032,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="245" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>93</v>
       </c>
@@ -21113,7 +21115,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="246" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A246" t="s">
         <v>93</v>
       </c>
@@ -21196,7 +21198,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="247" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
         <v>93</v>
       </c>
@@ -21860,7 +21862,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="255" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
         <v>95</v>
       </c>
@@ -21943,7 +21945,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="256" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A256" t="s">
         <v>95</v>
       </c>
@@ -22026,7 +22028,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="257" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
         <v>95</v>
       </c>
@@ -22109,7 +22111,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="258" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A258" t="s">
         <v>95</v>
       </c>
@@ -22773,7 +22775,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="266" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A266" t="s">
         <v>97</v>
       </c>
@@ -22856,7 +22858,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="267" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A267" t="s">
         <v>97</v>
       </c>
@@ -22939,7 +22941,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="268" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A268" t="s">
         <v>97</v>
       </c>
@@ -23022,7 +23024,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="269" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A269" t="s">
         <v>97</v>
       </c>
@@ -23686,7 +23688,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="277" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A277" t="s">
         <v>99</v>
       </c>
@@ -23769,7 +23771,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="278" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A278" t="s">
         <v>99</v>
       </c>
@@ -23852,7 +23854,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="279" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A279" t="s">
         <v>99</v>
       </c>
@@ -23935,7 +23937,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="280" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A280" t="s">
         <v>99</v>
       </c>
@@ -24599,7 +24601,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="288" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A288" t="s">
         <v>101</v>
       </c>
@@ -24682,7 +24684,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="289" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A289" t="s">
         <v>101</v>
       </c>
@@ -24765,7 +24767,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="290" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A290" t="s">
         <v>101</v>
       </c>
@@ -24848,7 +24850,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="291" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A291" t="s">
         <v>101</v>
       </c>
@@ -25512,7 +25514,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="299" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A299" t="s">
         <v>103</v>
       </c>
@@ -25595,7 +25597,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="300" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A300" t="s">
         <v>103</v>
       </c>
@@ -25678,7 +25680,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="301" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A301" t="s">
         <v>103</v>
       </c>
@@ -25761,7 +25763,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="302" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A302" t="s">
         <v>103</v>
       </c>
@@ -26425,7 +26427,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="310" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A310" t="s">
         <v>105</v>
       </c>
@@ -26508,7 +26510,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="311" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A311" t="s">
         <v>105</v>
       </c>
@@ -26591,7 +26593,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="312" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A312" t="s">
         <v>105</v>
       </c>
@@ -26674,7 +26676,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="313" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A313" t="s">
         <v>105</v>
       </c>
@@ -27338,7 +27340,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="321" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A321" t="s">
         <v>107</v>
       </c>
@@ -27421,7 +27423,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="322" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A322" t="s">
         <v>107</v>
       </c>
@@ -27504,7 +27506,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="323" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A323" t="s">
         <v>107</v>
       </c>
@@ -27587,7 +27589,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="324" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A324" t="s">
         <v>107</v>
       </c>
@@ -28253,17 +28255,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AB331" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="4">
-      <filters>
-        <filter val="EVI"/>
-        <filter val="NBR"/>
-        <filter val="NDVI"/>
-        <filter val="NDWI"/>
-        <filter val="SR_B5"/>
-        <filter val="SR_B6"/>
-        <filter val="SR_B7"/>
-      </filters>
-    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A6:AB331">
       <sortCondition ref="S1:S331"/>
     </sortState>

</xml_diff>